<commit_message>
Envoy 3.2: cool grey stone with copper, Traumsplitter instead of Äther
- Palette: cool grey stone instead of brown; copper stays as the warm
  accent, patina green and the pale glow of the shards for contrast;
  lighter text, copper eyebrows; textures, frames and the stone ledge
  are kept
- Currency renamed from Äther to Traumsplitter (key "splitter"), with a
  shard icon; Äther from older events still counts
- Items renamed to match: Nebelwickel, Splitterschale
- Map re-drawn less sepia: cool paper, distinct regions, copper
  mushrooms, patina shards in the Spalt; homes in grey stone with warm
  windows; app icon with a grey stone face; base figure in neutral grey
- Spec and CLAUDE.md updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0117M4aYJ5RoPwj7oU8m6XcB
</commit_message>
<xml_diff>
--- a/data/ausruestung.xlsx
+++ b/data/ausruestung.xlsx
@@ -1574,7 +1574,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>handschuhe_aetherwickel_4</t>
+          <t>handschuhe_nebelwickel_4</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1584,7 +1584,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Ätherwickel</t>
+          <t>Nebelwickel</t>
         </is>
       </c>
       <c r="D20" s="2" t="n">
@@ -1620,12 +1620,12 @@
       <c r="L20" s="2" t="inlineStr"/>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>handschuhe_aetherwickel_4.png</t>
+          <t>handschuhe_nebelwickel_4.png</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>icon_handschuhe_aetherwickel_4.png</t>
+          <t>icon_handschuhe_nebelwickel_4.png</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr"/>
@@ -1773,7 +1773,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Preis beim Händler in Äther. Leer = wird aus Stufe und Voraussetzungen berechnet.</t>
+          <t>Preis beim Händler in Traumsplittern. Leer = wird aus Stufe und Voraussetzungen berechnet.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Envoy 3.6: the Envoy is a woman, drawn by the user
Her drawings replace the placeholder figure: the base figure, the
starter outfit (Leinenhemd, Leinenhose) and the new Griffhandschuhe,
the reward for the bridge. The layers were cleaned of stray specks and
scaled to 1024 x 1536; the icons are cut free from the same drawings.

The starter outfit is worn from the start (herkunft 'angezogen').
All placeholder layers and item icons are gone: an item without a
picture is worn but not drawn, and shows the symbol of its slot. The
converter lists missing pictures as hints and leaves their path empty.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0117M4aYJ5RoPwj7oU8m6XcB
</commit_message>
<xml_diff>
--- a/data/ausruestung.xlsx
+++ b/data/ausruestung.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O20"/>
+  <dimension ref="A1:O21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -568,7 +568,7 @@
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>start, haendler</t>
+          <t>angezogen, haendler</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr"/>
@@ -619,7 +619,7 @@
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>start, haendler</t>
+          <t>angezogen, haendler</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr"/>
@@ -1043,7 +1043,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>handschuhe_lederwickel_2</t>
+          <t>handschuhe_griffhandschuhe_2</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1053,14 +1053,14 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Lederwickel</t>
+          <t>Griffhandschuhe</t>
         </is>
       </c>
       <c r="D11" s="2" t="n">
         <v>2</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F11" s="2" t="n">
         <v>0</v>
@@ -1073,28 +1073,28 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Schwerere Schläge, sicherer Griff.</t>
+          <t>Fester Griff, freie Finger.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>schaden:+2, treffer:+5</t>
+          <t>schaden:+2</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>haendler, beute</t>
+          <t>quest</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr"/>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>handschuhe_lederwickel_2.png</t>
+          <t>handschuhe_griffhandschuhe_2.png</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>icon_handschuhe_lederwickel_2.png</t>
+          <t>icon_handschuhe_griffhandschuhe_2.png</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr"/>
@@ -1102,42 +1102,42 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>kopf_kapuze_2</t>
+          <t>handschuhe_lederwickel_2</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>kopf</t>
+          <t>handschuhe</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Kapuze</t>
+          <t>Lederwickel</t>
         </is>
       </c>
       <c r="D12" s="2" t="n">
         <v>2</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F12" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Dämpft das Flüstern der Geister.</t>
+          <t>Schwerere Schläge, sicherer Griff.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>beruhigen:+8</t>
+          <t>schaden:+2, treffer:+5</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1148,12 +1148,12 @@
       <c r="L12" s="2" t="inlineStr"/>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>kopf_kapuze_2.png</t>
+          <t>handschuhe_lederwickel_2.png</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>icon_kopf_kapuze_2.png</t>
+          <t>icon_handschuhe_lederwickel_2.png</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr"/>
@@ -1161,17 +1161,17 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>umhang_nebelumhang_2</t>
+          <t>kopf_kapuze_2</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>umhang</t>
+          <t>kopf</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Nebelumhang</t>
+          <t>Kapuze</t>
         </is>
       </c>
       <c r="D13" s="2" t="n">
@@ -1184,35 +1184,35 @@
         <v>0</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Verschwimmt im Nebel.</t>
+          <t>Dämpft das Flüstern der Geister.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>ausweichen:+10</t>
+          <t>beruhigen:+8</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>beute</t>
+          <t>haendler, beute</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr"/>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>umhang_nebelumhang_2.png</t>
+          <t>kopf_kapuze_2.png</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>icon_umhang_nebelumhang_2.png</t>
+          <t>icon_kopf_kapuze_2.png</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr"/>
@@ -1220,58 +1220,58 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>torso_kampfjacke_3</t>
+          <t>umhang_nebelumhang_2</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>torso</t>
+          <t>umhang</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Gesteppte Kampfjacke</t>
+          <t>Nebelumhang</t>
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="F14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="G14" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="H14" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Hält auch schweren Treffern stand.</t>
+          <t>Verschwimmt im Nebel.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>ausweichen:+8, erholung:+5</t>
+          <t>ausweichen:+10</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>haendler, beute</t>
+          <t>beute</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr"/>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>torso_kampfjacke_3.png</t>
+          <t>umhang_nebelumhang_2.png</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>icon_torso_kampfjacke_3.png</t>
+          <t>icon_umhang_nebelumhang_2.png</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr"/>
@@ -1279,42 +1279,42 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>beine_wickelhose_3</t>
+          <t>torso_kampfjacke_3</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>beine</t>
+          <t>torso</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Wickelhose</t>
+          <t>Gesteppte Kampfjacke</t>
         </is>
       </c>
       <c r="D15" s="2" t="n">
         <v>3</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>Gebunden für schnelle Tritte.</t>
+          <t>Hält auch schweren Treffern stand.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>treffer:+8, ausweichen:+6</t>
+          <t>ausweichen:+8, erholung:+5</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1325,12 +1325,12 @@
       <c r="L15" s="2" t="inlineStr"/>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>beine_wickelhose_3.png</t>
+          <t>torso_kampfjacke_3.png</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>icon_beine_wickelhose_3.png</t>
+          <t>icon_torso_kampfjacke_3.png</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr"/>
@@ -1338,17 +1338,17 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>schuhe_leichtestiefel_3</t>
+          <t>beine_wickelhose_3</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>schuhe</t>
+          <t>beine</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Leichte Stiefel</t>
+          <t>Wickelhose</t>
         </is>
       </c>
       <c r="D16" s="2" t="n">
@@ -1358,38 +1358,38 @@
         <v>0</v>
       </c>
       <c r="F16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="G16" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" s="2" t="n">
-        <v>5</v>
-      </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Kaum zu hören, kaum zu spüren.</t>
+          <t>Gebunden für schnelle Tritte.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>reise:-2</t>
+          <t>treffer:+8, ausweichen:+6</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>quest</t>
+          <t>haendler, beute</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>schuhe_leichtestiefel_3.png</t>
+          <t>beine_wickelhose_3.png</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>icon_schuhe_leichtestiefel_3.png</t>
+          <t>icon_beine_wickelhose_3.png</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr"/>
@@ -1397,58 +1397,58 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>handschuhe_eisenwickel_3</t>
+          <t>schuhe_leichtestiefel_3</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>handschuhe</t>
+          <t>schuhe</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Eisenbeschlagene Wickel</t>
+          <t>Leichte Stiefel</t>
         </is>
       </c>
       <c r="D17" s="2" t="n">
         <v>3</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G17" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>Jeder Schlag sitzt.</t>
+          <t>Kaum zu hören, kaum zu spüren.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>schaden:+3, treffer:+5</t>
+          <t>reise:-2</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>haendler, beute</t>
+          <t>quest</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr"/>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>handschuhe_eisenwickel_3.png</t>
+          <t>schuhe_leichtestiefel_3.png</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>icon_handschuhe_eisenwickel_3.png</t>
+          <t>icon_schuhe_leichtestiefel_3.png</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr"/>
@@ -1456,58 +1456,58 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>kopf_stillemaske_3</t>
+          <t>handschuhe_eisenwickel_3</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>kopf</t>
+          <t>handschuhe</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Stille Maske</t>
+          <t>Eisenbeschlagene Wickel</t>
         </is>
       </c>
       <c r="D18" s="2" t="n">
         <v>3</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F18" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>Wer sie trägt, wird selbst still.</t>
+          <t>Jeder Schlag sitzt.</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>beruhigen:+15</t>
+          <t>schaden:+3, treffer:+5</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>quest</t>
+          <t>haendler, beute</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr"/>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>kopf_stillemaske_3.png</t>
+          <t>handschuhe_eisenwickel_3.png</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>icon_kopf_stillemaske_3.png</t>
+          <t>icon_handschuhe_eisenwickel_3.png</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr"/>
@@ -1515,17 +1515,17 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>umhang_sturmmantel_3</t>
+          <t>kopf_stillemaske_3</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>umhang</t>
+          <t>kopf</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Sturmmantel</t>
+          <t>Stille Maske</t>
         </is>
       </c>
       <c r="D19" s="2" t="n">
@@ -1535,38 +1535,38 @@
         <v>0</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H19" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>Trotzt jedem Wetter.</t>
+          <t>Wer sie trägt, wird selbst still.</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>ausweichen:+6, erholung:+8</t>
+          <t>beruhigen:+15</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>haendler, beute</t>
+          <t>quest</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr"/>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>umhang_sturmmantel_3.png</t>
+          <t>kopf_stillemaske_3.png</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>icon_umhang_sturmmantel_3.png</t>
+          <t>icon_kopf_stillemaske_3.png</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr"/>
@@ -1574,61 +1574,120 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>handschuhe_nebelwickel_4</t>
+          <t>umhang_sturmmantel_3</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>handschuhe</t>
+          <t>umhang</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Nebelwickel</t>
+          <t>Sturmmantel</t>
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H20" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>Werden kühl, wenn ein Geist nahe ist.</t>
+          <t>Trotzt jedem Wetter.</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>schaden:+4, beruhigen:+10</t>
+          <t>ausweichen:+6, erholung:+8</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>quest</t>
+          <t>haendler, beute</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr"/>
       <c r="M20" s="2" t="inlineStr">
         <is>
+          <t>umhang_sturmmantel_3.png</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>icon_umhang_sturmmantel_3.png</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>handschuhe_nebelwickel_4</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>handschuhe</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Nebelwickel</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>Werden kühl, wenn ein Geist nahe ist.</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>schaden:+4, beruhigen:+10</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>quest</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr"/>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
           <t>handschuhe_nebelwickel_4.png</t>
         </is>
       </c>
-      <c r="N20" s="2" t="inlineStr">
+      <c r="N21" s="2" t="inlineStr">
         <is>
           <t>icon_handschuhe_nebelwickel_4.png</t>
         </is>
       </c>
-      <c r="O20" s="2" t="inlineStr"/>
+      <c r="O21" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="2">
@@ -1761,7 +1820,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Wie man das Teil bekommt, mit Komma getrennt: start (im Rucksack beim Start), haendler, beute, quest.</t>
+          <t>Wie man das Teil bekommt, mit Komma getrennt: angezogen (trägt der Envoy von Anfang an), start (liegt beim Start im Rucksack), haendler, beute, quest.</t>
         </is>
       </c>
     </row>
@@ -1773,7 +1832,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Preis beim Händler in Traumsplittern. Leer = wird aus Stufe und Voraussetzungen berechnet.</t>
+          <t>Preis beim Händler in Bannsplittern. Leer = wird aus Stufe und Voraussetzungen berechnet.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Test folder before the real app, accessory slot, layer per item
Every push of the working branch now goes to a test folder next to the
real one (its name with -test). While uploading, that copy is marked as
the test version: it is called Envoy Test, shows a small Test sign and
keeps its browser data, offline store and server accounts apart from
the real app. Only the main branch goes to the real folder, and main
only gets what the user has looked at and released.

The cloak slot becomes Accessoire, a place for special things. Events
and tables with the old slot name still count. Each item may name
where its layer lies (column ebene), e.g. wide trousers over the shoes
or a shirt tucked in; the Kleiderkammer has the same field.

Content goes at most to a good midgame for now; noted in the docs.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0117M4aYJ5RoPwj7oU8m6XcB
</commit_message>
<xml_diff>
--- a/data/ausruestung.xlsx
+++ b/data/ausruestung.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O21"/>
+  <dimension ref="A1:P21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -453,7 +453,8 @@
     <col width="8" customWidth="1" min="12" max="12"/>
     <col width="34" customWidth="1" min="13" max="13"/>
     <col width="38" customWidth="1" min="14" max="14"/>
-    <col width="24" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="24" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -529,6 +530,11 @@
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
+          <t>ebene</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
           <t>notiz</t>
         </is>
       </c>
@@ -583,6 +589,7 @@
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr"/>
+      <c r="P2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -634,6 +641,7 @@
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr"/>
+      <c r="P3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -685,6 +693,7 @@
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr"/>
+      <c r="P4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -744,6 +753,7 @@
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr"/>
+      <c r="P5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -803,6 +813,7 @@
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr"/>
+      <c r="P6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -812,7 +823,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>umhang</t>
+          <t>accessoire</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -862,6 +873,7 @@
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr"/>
+      <c r="P7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -921,6 +933,7 @@
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr"/>
+      <c r="P8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -980,6 +993,7 @@
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr"/>
+      <c r="P9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1039,6 +1053,7 @@
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr"/>
+      <c r="P10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1098,6 +1113,7 @@
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr"/>
+      <c r="P11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1157,6 +1173,7 @@
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr"/>
+      <c r="P12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1216,6 +1233,7 @@
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr"/>
+      <c r="P13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1225,7 +1243,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>umhang</t>
+          <t>accessoire</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1275,6 +1293,7 @@
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr"/>
+      <c r="P14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1334,6 +1353,7 @@
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr"/>
+      <c r="P15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1393,6 +1413,7 @@
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr"/>
+      <c r="P16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1452,6 +1473,7 @@
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr"/>
+      <c r="P17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1511,6 +1533,7 @@
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr"/>
+      <c r="P18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1570,6 +1593,7 @@
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr"/>
+      <c r="P19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1579,7 +1603,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>umhang</t>
+          <t>accessoire</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1629,6 +1653,7 @@
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr"/>
+      <c r="P20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1688,11 +1713,15 @@
         </is>
       </c>
       <c r="O21" s="2" t="inlineStr"/>
+      <c r="P21" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"umhang,beine,schuhe,torso,handschuhe,kopf"</formula1>
+      <formula1>"accessoire,beine,schuhe,torso,handschuhe,kopf"</formula1>
+    </dataValidation>
+    <dataValidation sqref="O2:O500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Hinter der Figur,Unter der Hose,Über den Schuhen,Über jeder Hose,Unter dem Oberteil,Über dem Oberteil,Ganz vorn"</formula1>
     </dataValidation>
     <dataValidation sqref="E2:H500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="whole" operator="between">
       <formula1>0</formula1>
@@ -1709,7 +1738,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1748,7 +1777,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>umhang, beine, schuhe, torso, handschuhe oder kopf. Handschuhe sind die Wickel der waffenlosen Kampfkunst.</t>
+          <t>accessoire, beine, schuhe, torso, handschuhe oder kopf. Handschuhe sind die Wickel der waffenlosen Kampfkunst. Accessoire ist der Platz für Besonderes: Umhang, Schal, Tasche. Ältere Kennungen beginnen noch mit umhang_.</t>
         </is>
       </c>
     </row>
@@ -1863,10 +1892,22 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>ebene</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Wo das Bild liegt, wenn nicht am Platz seines Slots. Leer = wie der Slot. Hinten nach vorn: Hinter der Figur, (Figur), Unter der Hose, (Hose), (Schuhe), Über den Schuhen (weite Hose), Über jeder Hose (hohe Stiefel), Unter dem Oberteil, (Oberteil), Über dem Oberteil, (Hände), (Kopf), Ganz vorn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>notiz</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>Nur für dich, erscheint nicht in der App.</t>
         </is>

</xml_diff>

<commit_message>
Kleidung: viele Fundstücke in eigenen Farben
55 Teile aus der Kleiderkammer kommen ins Spiel, die meisten als Fund ohne
feste Quest: Auf Expeditionen und beim Sammeln findet der Envoy ab und zu
Kleidung (sicher spätestens nach 66 Energie, das erste Teil früh). Viele
Teile werden in einer von zwölf Farben gefunden; die App färbt Ebene und
Icon im Browser, Haut an Sandalen und Wickeln bleibt. Teile gelten für die
Frau, den Mann oder beide; was nicht zur Figur passt, wird weder gefunden
noch angeboten. Version 5.10.0.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0117M4aYJ5RoPwj7oU8m6XcB
</commit_message>
<xml_diff>
--- a/data/ausruestung.xlsx
+++ b/data/ausruestung.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P21"/>
+  <dimension ref="A1:R76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -454,7 +454,9 @@
     <col width="34" customWidth="1" min="13" max="13"/>
     <col width="38" customWidth="1" min="14" max="14"/>
     <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="24" customWidth="1" min="16" max="16"/>
+    <col width="9" customWidth="1" min="16" max="16"/>
+    <col width="9" customWidth="1" min="17" max="17"/>
+    <col width="24" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -535,6 +537,16 @@
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
+          <t>figur</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>faerbbar</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
           <t>notiz</t>
         </is>
       </c>
@@ -590,6 +602,8 @@
       </c>
       <c r="O2" s="2" t="inlineStr"/>
       <c r="P2" s="2" t="inlineStr"/>
+      <c r="Q2" s="2" t="inlineStr"/>
+      <c r="R2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -642,6 +656,8 @@
       </c>
       <c r="O3" s="2" t="inlineStr"/>
       <c r="P3" s="2" t="inlineStr"/>
+      <c r="Q3" s="2" t="inlineStr"/>
+      <c r="R3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -694,6 +710,8 @@
       </c>
       <c r="O4" s="2" t="inlineStr"/>
       <c r="P4" s="2" t="inlineStr"/>
+      <c r="Q4" s="2" t="inlineStr"/>
+      <c r="R4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -754,6 +772,8 @@
       </c>
       <c r="O5" s="2" t="inlineStr"/>
       <c r="P5" s="2" t="inlineStr"/>
+      <c r="Q5" s="2" t="inlineStr"/>
+      <c r="R5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -814,6 +834,8 @@
       </c>
       <c r="O6" s="2" t="inlineStr"/>
       <c r="P6" s="2" t="inlineStr"/>
+      <c r="Q6" s="2" t="inlineStr"/>
+      <c r="R6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -874,6 +896,8 @@
       </c>
       <c r="O7" s="2" t="inlineStr"/>
       <c r="P7" s="2" t="inlineStr"/>
+      <c r="Q7" s="2" t="inlineStr"/>
+      <c r="R7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -934,6 +958,8 @@
       </c>
       <c r="O8" s="2" t="inlineStr"/>
       <c r="P8" s="2" t="inlineStr"/>
+      <c r="Q8" s="2" t="inlineStr"/>
+      <c r="R8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -994,6 +1020,8 @@
       </c>
       <c r="O9" s="2" t="inlineStr"/>
       <c r="P9" s="2" t="inlineStr"/>
+      <c r="Q9" s="2" t="inlineStr"/>
+      <c r="R9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1054,6 +1082,8 @@
       </c>
       <c r="O10" s="2" t="inlineStr"/>
       <c r="P10" s="2" t="inlineStr"/>
+      <c r="Q10" s="2" t="inlineStr"/>
+      <c r="R10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1114,6 +1144,8 @@
       </c>
       <c r="O11" s="2" t="inlineStr"/>
       <c r="P11" s="2" t="inlineStr"/>
+      <c r="Q11" s="2" t="inlineStr"/>
+      <c r="R11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1174,6 +1206,8 @@
       </c>
       <c r="O12" s="2" t="inlineStr"/>
       <c r="P12" s="2" t="inlineStr"/>
+      <c r="Q12" s="2" t="inlineStr"/>
+      <c r="R12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1234,6 +1268,8 @@
       </c>
       <c r="O13" s="2" t="inlineStr"/>
       <c r="P13" s="2" t="inlineStr"/>
+      <c r="Q13" s="2" t="inlineStr"/>
+      <c r="R13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1294,6 +1330,8 @@
       </c>
       <c r="O14" s="2" t="inlineStr"/>
       <c r="P14" s="2" t="inlineStr"/>
+      <c r="Q14" s="2" t="inlineStr"/>
+      <c r="R14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1354,6 +1392,8 @@
       </c>
       <c r="O15" s="2" t="inlineStr"/>
       <c r="P15" s="2" t="inlineStr"/>
+      <c r="Q15" s="2" t="inlineStr"/>
+      <c r="R15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1414,6 +1454,8 @@
       </c>
       <c r="O16" s="2" t="inlineStr"/>
       <c r="P16" s="2" t="inlineStr"/>
+      <c r="Q16" s="2" t="inlineStr"/>
+      <c r="R16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1474,6 +1516,8 @@
       </c>
       <c r="O17" s="2" t="inlineStr"/>
       <c r="P17" s="2" t="inlineStr"/>
+      <c r="Q17" s="2" t="inlineStr"/>
+      <c r="R17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1534,6 +1578,8 @@
       </c>
       <c r="O18" s="2" t="inlineStr"/>
       <c r="P18" s="2" t="inlineStr"/>
+      <c r="Q18" s="2" t="inlineStr"/>
+      <c r="R18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1594,6 +1640,8 @@
       </c>
       <c r="O19" s="2" t="inlineStr"/>
       <c r="P19" s="2" t="inlineStr"/>
+      <c r="Q19" s="2" t="inlineStr"/>
+      <c r="R19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1654,6 +1702,8 @@
       </c>
       <c r="O20" s="2" t="inlineStr"/>
       <c r="P20" s="2" t="inlineStr"/>
+      <c r="Q20" s="2" t="inlineStr"/>
+      <c r="R20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1714,14 +1764,3664 @@
       </c>
       <c r="O21" s="2" t="inlineStr"/>
       <c r="P21" s="2" t="inlineStr"/>
+      <c r="Q21" s="2" t="inlineStr"/>
+      <c r="R21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>beine_stoffhose_1</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>beine</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Stoffhose</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr"/>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>beine_stoffhose_1.png</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>icon_beine_stoffhose_1.png</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr"/>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>beide</t>
+        </is>
+      </c>
+      <c r="Q22" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R22" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 14, 68</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>beine_zweifarbigepumphose_2</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>beine</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Zweifarbige Pumphose</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I23" s="2" t="inlineStr"/>
+      <c r="J23" s="2" t="inlineStr"/>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr"/>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>beine_zweifarbigepumphose_2.png</t>
+        </is>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>icon_beine_zweifarbigepumphose_2.png</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr"/>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>beide</t>
+        </is>
+      </c>
+      <c r="Q23" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R23" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 15</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>beine_bundhose_1</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>beine</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Bundhose</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr"/>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr"/>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>beine_bundhose_1.png</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>icon_beine_bundhose_1.png</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr"/>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>beide</t>
+        </is>
+      </c>
+      <c r="Q24" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R24" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 16, 72</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>beine_pumphose_2</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>beine</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Pumphose</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" s="2" t="inlineStr"/>
+      <c r="J25" s="2" t="inlineStr"/>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr"/>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>beine_pumphose_2.png</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>icon_beine_pumphose_2.png</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr"/>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>beide</t>
+        </is>
+      </c>
+      <c r="Q25" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R25" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 17, 69</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>beine_schaerpenhose_2</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>beine</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Schärpenhose</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I26" s="2" t="inlineStr"/>
+      <c r="J26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr"/>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>beine_schaerpenhose_2.png</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>icon_beine_schaerpenhose_2.png</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>Über den Schuhen</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>beide</t>
+        </is>
+      </c>
+      <c r="Q26" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R26" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 18, 71</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>beine_flickenhose_2</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>beine</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Flickenhose</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" s="2" t="inlineStr"/>
+      <c r="J27" s="2" t="inlineStr"/>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr"/>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>beine_flickenhose_2.png</t>
+        </is>
+      </c>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>icon_beine_flickenhose_2.png</t>
+        </is>
+      </c>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>Über den Schuhen</t>
+        </is>
+      </c>
+      <c r="P27" s="2" t="inlineStr">
+        <is>
+          <t>beide</t>
+        </is>
+      </c>
+      <c r="Q27" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R27" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 19, 67</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>beine_bunteflickenhose_2</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>beine</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Bunte Flickenhose</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E28" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" s="2" t="inlineStr"/>
+      <c r="J28" s="2" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr"/>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>beine_bunteflickenhose_2.png</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>icon_beine_bunteflickenhose_2.png</t>
+        </is>
+      </c>
+      <c r="O28" s="2" t="inlineStr"/>
+      <c r="P28" s="2" t="inlineStr">
+        <is>
+          <t>beide</t>
+        </is>
+      </c>
+      <c r="Q28" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R28" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 20, 70</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>beine_blaetterleggings_2</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>beine</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Blätterleggings</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I29" s="2" t="inlineStr"/>
+      <c r="J29" s="2" t="inlineStr"/>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr"/>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>beine_blaetterleggings_2.png</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>icon_beine_blaetterleggings_2.png</t>
+        </is>
+      </c>
+      <c r="O29" s="2" t="inlineStr"/>
+      <c r="P29" s="2" t="inlineStr">
+        <is>
+          <t>Frau</t>
+        </is>
+      </c>
+      <c r="Q29" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R29" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 21</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>beine_musterleggings_2</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>beine</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Musterleggings</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" s="2" t="inlineStr"/>
+      <c r="J30" s="2" t="inlineStr"/>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr"/>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>beine_musterleggings_2.png</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>icon_beine_musterleggings_2.png</t>
+        </is>
+      </c>
+      <c r="O30" s="2" t="inlineStr"/>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>Frau</t>
+        </is>
+      </c>
+      <c r="Q30" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R30" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 22</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>beine_wanderhose_2</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>beine</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Wanderhose</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" s="2" t="inlineStr"/>
+      <c r="J31" s="2" t="inlineStr"/>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr"/>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>beine_wanderhose_2.png</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>icon_beine_wanderhose_2.png</t>
+        </is>
+      </c>
+      <c r="O31" s="2" t="inlineStr"/>
+      <c r="P31" s="2" t="inlineStr">
+        <is>
+          <t>beide</t>
+        </is>
+      </c>
+      <c r="Q31" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R31" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 23</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>beine_kurzehose_1</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>beine</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Kurze Hose</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" s="2" t="inlineStr"/>
+      <c r="J32" s="2" t="inlineStr"/>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr"/>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>beine_kurzehose_1.png</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>icon_beine_kurzehose_1.png</t>
+        </is>
+      </c>
+      <c r="O32" s="2" t="inlineStr"/>
+      <c r="P32" s="2" t="inlineStr">
+        <is>
+          <t>Frau</t>
+        </is>
+      </c>
+      <c r="Q32" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R32" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 24</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>beine_engejeans_1</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>beine</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Enge Jeans</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I33" s="2" t="inlineStr"/>
+      <c r="J33" s="2" t="inlineStr"/>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr"/>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>beine_engejeans_1.png</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>icon_beine_engejeans_1.png</t>
+        </is>
+      </c>
+      <c r="O33" s="2" t="inlineStr"/>
+      <c r="P33" s="2" t="inlineStr">
+        <is>
+          <t>Frau</t>
+        </is>
+      </c>
+      <c r="Q33" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R33" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 25</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>beine_weitejeans_1</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>beine</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Weite Jeans</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" s="2" t="inlineStr"/>
+      <c r="J34" s="2" t="inlineStr"/>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr"/>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>beine_weitejeans_1.png</t>
+        </is>
+      </c>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>icon_beine_weitejeans_1.png</t>
+        </is>
+      </c>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>Über den Schuhen</t>
+        </is>
+      </c>
+      <c r="P34" s="2" t="inlineStr">
+        <is>
+          <t>beide</t>
+        </is>
+      </c>
+      <c r="Q34" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R34" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 26</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>beine_jeansmitbuendchen_2</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>beine</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Jeans mit Bündchen</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I35" s="2" t="inlineStr"/>
+      <c r="J35" s="2" t="inlineStr"/>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="inlineStr"/>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>beine_jeansmitbuendchen_2.png</t>
+        </is>
+      </c>
+      <c r="N35" s="2" t="inlineStr">
+        <is>
+          <t>icon_beine_jeansmitbuendchen_2.png</t>
+        </is>
+      </c>
+      <c r="O35" s="2" t="inlineStr"/>
+      <c r="P35" s="2" t="inlineStr">
+        <is>
+          <t>beide</t>
+        </is>
+      </c>
+      <c r="Q35" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R35" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 27</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>beine_leggings_1</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>beine</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Leggings</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" s="2" t="inlineStr"/>
+      <c r="J36" s="2" t="inlineStr"/>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr"/>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>beine_leggings_1.png</t>
+        </is>
+      </c>
+      <c r="N36" s="2" t="inlineStr">
+        <is>
+          <t>icon_beine_leggings_1.png</t>
+        </is>
+      </c>
+      <c r="O36" s="2" t="inlineStr"/>
+      <c r="P36" s="2" t="inlineStr">
+        <is>
+          <t>Frau</t>
+        </is>
+      </c>
+      <c r="Q36" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R36" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 28</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>beine_cargohose_3</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>beine</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Cargohose</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E37" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I37" s="2" t="inlineStr"/>
+      <c r="J37" s="2" t="inlineStr"/>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="inlineStr"/>
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>beine_cargohose_3.png</t>
+        </is>
+      </c>
+      <c r="N37" s="2" t="inlineStr">
+        <is>
+          <t>icon_beine_cargohose_3.png</t>
+        </is>
+      </c>
+      <c r="O37" s="2" t="inlineStr"/>
+      <c r="P37" s="2" t="inlineStr">
+        <is>
+          <t>beide</t>
+        </is>
+      </c>
+      <c r="Q37" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R37" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 29</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>beine_hosenrock_3</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>beine</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Hosenrock</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I38" s="2" t="inlineStr"/>
+      <c r="J38" s="2" t="inlineStr"/>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr"/>
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>beine_hosenrock_3.png</t>
+        </is>
+      </c>
+      <c r="N38" s="2" t="inlineStr">
+        <is>
+          <t>icon_beine_hosenrock_3.png</t>
+        </is>
+      </c>
+      <c r="O38" s="2" t="inlineStr"/>
+      <c r="P38" s="2" t="inlineStr">
+        <is>
+          <t>Frau</t>
+        </is>
+      </c>
+      <c r="Q38" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R38" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>torso_bergpulli_2</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>torso</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Bergpulli</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" s="2" t="inlineStr"/>
+      <c r="J39" s="2" t="inlineStr"/>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L39" s="2" t="inlineStr"/>
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>torso_bergpulli_2.png</t>
+        </is>
+      </c>
+      <c r="N39" s="2" t="inlineStr">
+        <is>
+          <t>icon_torso_bergpulli_2.png</t>
+        </is>
+      </c>
+      <c r="O39" s="2" t="inlineStr"/>
+      <c r="P39" s="2" t="inlineStr">
+        <is>
+          <t>Frau</t>
+        </is>
+      </c>
+      <c r="Q39" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R39" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 31</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>torso_druckshirt_1</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>torso</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Druckshirt</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I40" s="2" t="inlineStr"/>
+      <c r="J40" s="2" t="inlineStr"/>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="inlineStr"/>
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>torso_druckshirt_1.png</t>
+        </is>
+      </c>
+      <c r="N40" s="2" t="inlineStr">
+        <is>
+          <t>icon_torso_druckshirt_1.png</t>
+        </is>
+      </c>
+      <c r="O40" s="2" t="inlineStr"/>
+      <c r="P40" s="2" t="inlineStr">
+        <is>
+          <t>beide</t>
+        </is>
+      </c>
+      <c r="Q40" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R40" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 32, 86</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>torso_mosaiktop_2</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>torso</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Mosaik-Top</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I41" s="2" t="inlineStr"/>
+      <c r="J41" s="2" t="inlineStr"/>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L41" s="2" t="inlineStr"/>
+      <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>torso_mosaiktop_2.png</t>
+        </is>
+      </c>
+      <c r="N41" s="2" t="inlineStr">
+        <is>
+          <t>icon_torso_mosaiktop_2.png</t>
+        </is>
+      </c>
+      <c r="O41" s="2" t="inlineStr"/>
+      <c r="P41" s="2" t="inlineStr">
+        <is>
+          <t>Frau</t>
+        </is>
+      </c>
+      <c r="Q41" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R41" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 33</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>torso_stickereitop_2</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>torso</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Stickerei-Top</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" s="2" t="inlineStr"/>
+      <c r="J42" s="2" t="inlineStr"/>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr"/>
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>torso_stickereitop_2.png</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="inlineStr">
+        <is>
+          <t>icon_torso_stickereitop_2.png</t>
+        </is>
+      </c>
+      <c r="O42" s="2" t="inlineStr"/>
+      <c r="P42" s="2" t="inlineStr">
+        <is>
+          <t>Frau</t>
+        </is>
+      </c>
+      <c r="Q42" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R42" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 34</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>torso_bestickterbolero_3</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>torso</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Bestickter Bolero</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="I43" s="2" t="inlineStr"/>
+      <c r="J43" s="2" t="inlineStr"/>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L43" s="2" t="inlineStr"/>
+      <c r="M43" s="2" t="inlineStr">
+        <is>
+          <t>torso_bestickterbolero_3.png</t>
+        </is>
+      </c>
+      <c r="N43" s="2" t="inlineStr">
+        <is>
+          <t>icon_torso_bestickterbolero_3.png</t>
+        </is>
+      </c>
+      <c r="O43" s="2" t="inlineStr"/>
+      <c r="P43" s="2" t="inlineStr">
+        <is>
+          <t>Frau</t>
+        </is>
+      </c>
+      <c r="Q43" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R43" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 35</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>torso_schlichtesshirt_1</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>torso</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Schlichtes Shirt</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I44" s="2" t="inlineStr"/>
+      <c r="J44" s="2" t="inlineStr"/>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L44" s="2" t="inlineStr"/>
+      <c r="M44" s="2" t="inlineStr">
+        <is>
+          <t>torso_schlichtesshirt_1.png</t>
+        </is>
+      </c>
+      <c r="N44" s="2" t="inlineStr">
+        <is>
+          <t>icon_torso_schlichtesshirt_1.png</t>
+        </is>
+      </c>
+      <c r="O44" s="2" t="inlineStr"/>
+      <c r="P44" s="2" t="inlineStr">
+        <is>
+          <t>beide</t>
+        </is>
+      </c>
+      <c r="Q44" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R44" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 36, 76</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>torso_lederwams_3</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>torso</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Lederwams</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E45" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="F45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I45" s="2" t="inlineStr"/>
+      <c r="J45" s="2" t="inlineStr"/>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L45" s="2" t="inlineStr"/>
+      <c r="M45" s="2" t="inlineStr">
+        <is>
+          <t>torso_lederwams_3.png</t>
+        </is>
+      </c>
+      <c r="N45" s="2" t="inlineStr">
+        <is>
+          <t>icon_torso_lederwams_3.png</t>
+        </is>
+      </c>
+      <c r="O45" s="2" t="inlineStr"/>
+      <c r="P45" s="2" t="inlineStr">
+        <is>
+          <t>Frau</t>
+        </is>
+      </c>
+      <c r="Q45" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R45" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 37</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>torso_rautenpulli_2</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>torso</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Rautenpulli</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="G46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I46" s="2" t="inlineStr"/>
+      <c r="J46" s="2" t="inlineStr"/>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L46" s="2" t="inlineStr"/>
+      <c r="M46" s="2" t="inlineStr">
+        <is>
+          <t>torso_rautenpulli_2.png</t>
+        </is>
+      </c>
+      <c r="N46" s="2" t="inlineStr">
+        <is>
+          <t>icon_torso_rautenpulli_2.png</t>
+        </is>
+      </c>
+      <c r="O46" s="2" t="inlineStr"/>
+      <c r="P46" s="2" t="inlineStr">
+        <is>
+          <t>Frau</t>
+        </is>
+      </c>
+      <c r="Q46" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R46" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 38</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>torso_lagentop_1</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>torso</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Lagen-Top</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I47" s="2" t="inlineStr"/>
+      <c r="J47" s="2" t="inlineStr"/>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L47" s="2" t="inlineStr"/>
+      <c r="M47" s="2" t="inlineStr">
+        <is>
+          <t>torso_lagentop_1.png</t>
+        </is>
+      </c>
+      <c r="N47" s="2" t="inlineStr">
+        <is>
+          <t>icon_torso_lagentop_1.png</t>
+        </is>
+      </c>
+      <c r="O47" s="2" t="inlineStr"/>
+      <c r="P47" s="2" t="inlineStr">
+        <is>
+          <t>Frau</t>
+        </is>
+      </c>
+      <c r="Q47" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R47" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 39</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>torso_norwegerhoodie_2</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>torso</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Norweger-Hoodie</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I48" s="2" t="inlineStr"/>
+      <c r="J48" s="2" t="inlineStr"/>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L48" s="2" t="inlineStr"/>
+      <c r="M48" s="2" t="inlineStr">
+        <is>
+          <t>torso_norwegerhoodie_2.png</t>
+        </is>
+      </c>
+      <c r="N48" s="2" t="inlineStr">
+        <is>
+          <t>icon_torso_norwegerhoodie_2.png</t>
+        </is>
+      </c>
+      <c r="O48" s="2" t="inlineStr"/>
+      <c r="P48" s="2" t="inlineStr">
+        <is>
+          <t>beide</t>
+        </is>
+      </c>
+      <c r="Q48" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R48" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 40, 84</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>torso_grobstrickpulli_2</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>torso</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Grobstrickpulli</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I49" s="2" t="inlineStr"/>
+      <c r="J49" s="2" t="inlineStr"/>
+      <c r="K49" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L49" s="2" t="inlineStr"/>
+      <c r="M49" s="2" t="inlineStr">
+        <is>
+          <t>torso_grobstrickpulli_2.png</t>
+        </is>
+      </c>
+      <c r="N49" s="2" t="inlineStr">
+        <is>
+          <t>icon_torso_grobstrickpulli_2.png</t>
+        </is>
+      </c>
+      <c r="O49" s="2" t="inlineStr"/>
+      <c r="P49" s="2" t="inlineStr">
+        <is>
+          <t>Frau</t>
+        </is>
+      </c>
+      <c r="Q49" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R49" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 41</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>torso_leinenbluse_1</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>torso</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Leinenbluse</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I50" s="2" t="inlineStr"/>
+      <c r="J50" s="2" t="inlineStr"/>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L50" s="2" t="inlineStr"/>
+      <c r="M50" s="2" t="inlineStr">
+        <is>
+          <t>torso_leinenbluse_1.png</t>
+        </is>
+      </c>
+      <c r="N50" s="2" t="inlineStr">
+        <is>
+          <t>icon_torso_leinenbluse_1.png</t>
+        </is>
+      </c>
+      <c r="O50" s="2" t="inlineStr"/>
+      <c r="P50" s="2" t="inlineStr">
+        <is>
+          <t>Frau</t>
+        </is>
+      </c>
+      <c r="Q50" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R50" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 42</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>torso_sonnenshirt_1</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>torso</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Sonnenshirt</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I51" s="2" t="inlineStr"/>
+      <c r="J51" s="2" t="inlineStr"/>
+      <c r="K51" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L51" s="2" t="inlineStr"/>
+      <c r="M51" s="2" t="inlineStr">
+        <is>
+          <t>torso_sonnenshirt_1.png</t>
+        </is>
+      </c>
+      <c r="N51" s="2" t="inlineStr">
+        <is>
+          <t>icon_torso_sonnenshirt_1.png</t>
+        </is>
+      </c>
+      <c r="O51" s="2" t="inlineStr"/>
+      <c r="P51" s="2" t="inlineStr">
+        <is>
+          <t>Frau</t>
+        </is>
+      </c>
+      <c r="Q51" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R51" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 43</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>torso_baenderpulli_2</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>torso</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Bänderpulli</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H52" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="I52" s="2" t="inlineStr"/>
+      <c r="J52" s="2" t="inlineStr"/>
+      <c r="K52" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L52" s="2" t="inlineStr"/>
+      <c r="M52" s="2" t="inlineStr">
+        <is>
+          <t>torso_baenderpulli_2.png</t>
+        </is>
+      </c>
+      <c r="N52" s="2" t="inlineStr">
+        <is>
+          <t>icon_torso_baenderpulli_2.png</t>
+        </is>
+      </c>
+      <c r="O52" s="2" t="inlineStr"/>
+      <c r="P52" s="2" t="inlineStr">
+        <is>
+          <t>Frau</t>
+        </is>
+      </c>
+      <c r="Q52" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R52" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 44</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>torso_langarmshirt_1</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>torso</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Langarmshirt</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I53" s="2" t="inlineStr"/>
+      <c r="J53" s="2" t="inlineStr"/>
+      <c r="K53" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L53" s="2" t="inlineStr"/>
+      <c r="M53" s="2" t="inlineStr">
+        <is>
+          <t>torso_langarmshirt_1.png</t>
+        </is>
+      </c>
+      <c r="N53" s="2" t="inlineStr">
+        <is>
+          <t>icon_torso_langarmshirt_1.png</t>
+        </is>
+      </c>
+      <c r="O53" s="2" t="inlineStr"/>
+      <c r="P53" s="2" t="inlineStr">
+        <is>
+          <t>Frau</t>
+        </is>
+      </c>
+      <c r="Q53" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R53" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 46</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>torso_besticktetunika_3</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>torso</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Bestickte Tunika</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G54" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I54" s="2" t="inlineStr"/>
+      <c r="J54" s="2" t="inlineStr"/>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L54" s="2" t="inlineStr"/>
+      <c r="M54" s="2" t="inlineStr">
+        <is>
+          <t>torso_besticktetunika_3.png</t>
+        </is>
+      </c>
+      <c r="N54" s="2" t="inlineStr">
+        <is>
+          <t>icon_torso_besticktetunika_3.png</t>
+        </is>
+      </c>
+      <c r="O54" s="2" t="inlineStr"/>
+      <c r="P54" s="2" t="inlineStr">
+        <is>
+          <t>beide</t>
+        </is>
+      </c>
+      <c r="Q54" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R54" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 47, 73</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>torso_sportshirt_2</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>torso</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Sportshirt</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F55" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I55" s="2" t="inlineStr"/>
+      <c r="J55" s="2" t="inlineStr"/>
+      <c r="K55" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L55" s="2" t="inlineStr"/>
+      <c r="M55" s="2" t="inlineStr">
+        <is>
+          <t>torso_sportshirt_2.png</t>
+        </is>
+      </c>
+      <c r="N55" s="2" t="inlineStr">
+        <is>
+          <t>icon_torso_sportshirt_2.png</t>
+        </is>
+      </c>
+      <c r="O55" s="2" t="inlineStr"/>
+      <c r="P55" s="2" t="inlineStr">
+        <is>
+          <t>beide</t>
+        </is>
+      </c>
+      <c r="Q55" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R55" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 48, 82</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>torso_zackenshirt_2</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>torso</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Zackenshirt</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E56" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I56" s="2" t="inlineStr"/>
+      <c r="J56" s="2" t="inlineStr"/>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L56" s="2" t="inlineStr"/>
+      <c r="M56" s="2" t="inlineStr">
+        <is>
+          <t>torso_zackenshirt_2.png</t>
+        </is>
+      </c>
+      <c r="N56" s="2" t="inlineStr">
+        <is>
+          <t>icon_torso_zackenshirt_2.png</t>
+        </is>
+      </c>
+      <c r="O56" s="2" t="inlineStr"/>
+      <c r="P56" s="2" t="inlineStr">
+        <is>
+          <t>Frau</t>
+        </is>
+      </c>
+      <c r="Q56" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R56" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 49</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>torso_turnanzug_3</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>torso</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Turnanzug</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E57" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F57" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G57" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H57" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="I57" s="2" t="inlineStr"/>
+      <c r="J57" s="2" t="inlineStr"/>
+      <c r="K57" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L57" s="2" t="inlineStr"/>
+      <c r="M57" s="2" t="inlineStr">
+        <is>
+          <t>torso_turnanzug_3.png</t>
+        </is>
+      </c>
+      <c r="N57" s="2" t="inlineStr">
+        <is>
+          <t>icon_torso_turnanzug_3.png</t>
+        </is>
+      </c>
+      <c r="O57" s="2" t="inlineStr"/>
+      <c r="P57" s="2" t="inlineStr">
+        <is>
+          <t>Frau</t>
+        </is>
+      </c>
+      <c r="Q57" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R57" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 50</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>torso_knopfshirt_1</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>torso</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Knopfshirt</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I58" s="2" t="inlineStr"/>
+      <c r="J58" s="2" t="inlineStr"/>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L58" s="2" t="inlineStr"/>
+      <c r="M58" s="2" t="inlineStr">
+        <is>
+          <t>torso_knopfshirt_1.png</t>
+        </is>
+      </c>
+      <c r="N58" s="2" t="inlineStr">
+        <is>
+          <t>icon_torso_knopfshirt_1.png</t>
+        </is>
+      </c>
+      <c r="O58" s="2" t="inlineStr"/>
+      <c r="P58" s="2" t="inlineStr">
+        <is>
+          <t>beide</t>
+        </is>
+      </c>
+      <c r="Q58" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R58" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 51, 75</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>torso_baseballshirt_2</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>torso</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Baseballshirt</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E59" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I59" s="2" t="inlineStr"/>
+      <c r="J59" s="2" t="inlineStr"/>
+      <c r="K59" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L59" s="2" t="inlineStr"/>
+      <c r="M59" s="2" t="inlineStr">
+        <is>
+          <t>torso_baseballshirt_2.png</t>
+        </is>
+      </c>
+      <c r="N59" s="2" t="inlineStr">
+        <is>
+          <t>icon_torso_baseballshirt_2.png</t>
+        </is>
+      </c>
+      <c r="O59" s="2" t="inlineStr"/>
+      <c r="P59" s="2" t="inlineStr">
+        <is>
+          <t>Frau</t>
+        </is>
+      </c>
+      <c r="Q59" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R59" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 55</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>torso_sporttop_2</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>torso</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Sport-Top</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F60" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="G60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I60" s="2" t="inlineStr"/>
+      <c r="J60" s="2" t="inlineStr"/>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L60" s="2" t="inlineStr"/>
+      <c r="M60" s="2" t="inlineStr">
+        <is>
+          <t>torso_sporttop_2.png</t>
+        </is>
+      </c>
+      <c r="N60" s="2" t="inlineStr">
+        <is>
+          <t>icon_torso_sporttop_2.png</t>
+        </is>
+      </c>
+      <c r="O60" s="2" t="inlineStr"/>
+      <c r="P60" s="2" t="inlineStr">
+        <is>
+          <t>Frau</t>
+        </is>
+      </c>
+      <c r="Q60" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R60" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 56</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>torso_wickelbluse_2</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>torso</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>Wickelbluse</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E61" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F61" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G61" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H61" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="I61" s="2" t="inlineStr"/>
+      <c r="J61" s="2" t="inlineStr"/>
+      <c r="K61" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L61" s="2" t="inlineStr"/>
+      <c r="M61" s="2" t="inlineStr">
+        <is>
+          <t>torso_wickelbluse_2.png</t>
+        </is>
+      </c>
+      <c r="N61" s="2" t="inlineStr">
+        <is>
+          <t>icon_torso_wickelbluse_2.png</t>
+        </is>
+      </c>
+      <c r="O61" s="2" t="inlineStr"/>
+      <c r="P61" s="2" t="inlineStr">
+        <is>
+          <t>Frau</t>
+        </is>
+      </c>
+      <c r="Q61" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R61" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 57</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>torso_batikshirt_2</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>torso</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Batikshirt</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E62" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F62" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G62" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H62" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I62" s="2" t="inlineStr"/>
+      <c r="J62" s="2" t="inlineStr"/>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L62" s="2" t="inlineStr"/>
+      <c r="M62" s="2" t="inlineStr">
+        <is>
+          <t>torso_batikshirt_2.png</t>
+        </is>
+      </c>
+      <c r="N62" s="2" t="inlineStr">
+        <is>
+          <t>icon_torso_batikshirt_2.png</t>
+        </is>
+      </c>
+      <c r="O62" s="2" t="inlineStr"/>
+      <c r="P62" s="2" t="inlineStr">
+        <is>
+          <t>beide</t>
+        </is>
+      </c>
+      <c r="Q62" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R62" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 58, 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>torso_raglanshirt_1</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>torso</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>Raglanshirt</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E63" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F63" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G63" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H63" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I63" s="2" t="inlineStr"/>
+      <c r="J63" s="2" t="inlineStr"/>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L63" s="2" t="inlineStr"/>
+      <c r="M63" s="2" t="inlineStr">
+        <is>
+          <t>torso_raglanshirt_1.png</t>
+        </is>
+      </c>
+      <c r="N63" s="2" t="inlineStr">
+        <is>
+          <t>icon_torso_raglanshirt_1.png</t>
+        </is>
+      </c>
+      <c r="O63" s="2" t="inlineStr"/>
+      <c r="P63" s="2" t="inlineStr">
+        <is>
+          <t>beide</t>
+        </is>
+      </c>
+      <c r="Q63" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R63" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 59, 80</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>torso_ringelshirt_1</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>torso</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>Ringelshirt</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E64" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F64" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G64" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H64" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I64" s="2" t="inlineStr"/>
+      <c r="J64" s="2" t="inlineStr"/>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L64" s="2" t="inlineStr"/>
+      <c r="M64" s="2" t="inlineStr">
+        <is>
+          <t>torso_ringelshirt_1.png</t>
+        </is>
+      </c>
+      <c r="N64" s="2" t="inlineStr">
+        <is>
+          <t>icon_torso_ringelshirt_1.png</t>
+        </is>
+      </c>
+      <c r="O64" s="2" t="inlineStr"/>
+      <c r="P64" s="2" t="inlineStr">
+        <is>
+          <t>Frau</t>
+        </is>
+      </c>
+      <c r="Q64" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R64" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 60</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>torso_katzenshirt_2</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>torso</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>Katzenshirt</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E65" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F65" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G65" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H65" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I65" s="2" t="inlineStr"/>
+      <c r="J65" s="2" t="inlineStr"/>
+      <c r="K65" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L65" s="2" t="inlineStr"/>
+      <c r="M65" s="2" t="inlineStr">
+        <is>
+          <t>torso_katzenshirt_2.png</t>
+        </is>
+      </c>
+      <c r="N65" s="2" t="inlineStr">
+        <is>
+          <t>icon_torso_katzenshirt_2.png</t>
+        </is>
+      </c>
+      <c r="O65" s="2" t="inlineStr"/>
+      <c r="P65" s="2" t="inlineStr">
+        <is>
+          <t>beide</t>
+        </is>
+      </c>
+      <c r="Q65" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R65" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 61, 87</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>torso_waldshirt_3</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>torso</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Waldshirt</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E66" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F66" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G66" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H66" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I66" s="2" t="inlineStr"/>
+      <c r="J66" s="2" t="inlineStr"/>
+      <c r="K66" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L66" s="2" t="inlineStr"/>
+      <c r="M66" s="2" t="inlineStr">
+        <is>
+          <t>torso_waldshirt_3.png</t>
+        </is>
+      </c>
+      <c r="N66" s="2" t="inlineStr">
+        <is>
+          <t>icon_torso_waldshirt_3.png</t>
+        </is>
+      </c>
+      <c r="O66" s="2" t="inlineStr"/>
+      <c r="P66" s="2" t="inlineStr">
+        <is>
+          <t>Frau</t>
+        </is>
+      </c>
+      <c r="Q66" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R66" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 62</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>torso_weitesshirt_1</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>torso</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Weites Shirt</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E67" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F67" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G67" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H67" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I67" s="2" t="inlineStr"/>
+      <c r="J67" s="2" t="inlineStr"/>
+      <c r="K67" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L67" s="2" t="inlineStr"/>
+      <c r="M67" s="2" t="inlineStr">
+        <is>
+          <t>torso_weitesshirt_1.png</t>
+        </is>
+      </c>
+      <c r="N67" s="2" t="inlineStr">
+        <is>
+          <t>icon_torso_weitesshirt_1.png</t>
+        </is>
+      </c>
+      <c r="O67" s="2" t="inlineStr"/>
+      <c r="P67" s="2" t="inlineStr">
+        <is>
+          <t>beide</t>
+        </is>
+      </c>
+      <c r="Q67" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R67" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 63, 83</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>torso_bandshirt_2</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>torso</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Bandshirt</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E68" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I68" s="2" t="inlineStr"/>
+      <c r="J68" s="2" t="inlineStr"/>
+      <c r="K68" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L68" s="2" t="inlineStr"/>
+      <c r="M68" s="2" t="inlineStr">
+        <is>
+          <t>torso_bandshirt_2.png</t>
+        </is>
+      </c>
+      <c r="N68" s="2" t="inlineStr">
+        <is>
+          <t>icon_torso_bandshirt_2.png</t>
+        </is>
+      </c>
+      <c r="O68" s="2" t="inlineStr"/>
+      <c r="P68" s="2" t="inlineStr">
+        <is>
+          <t>beide</t>
+        </is>
+      </c>
+      <c r="Q68" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R68" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 64, 77</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>torso_haekelshirt_3</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>torso</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>Häkelshirt</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H69" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="I69" s="2" t="inlineStr"/>
+      <c r="J69" s="2" t="inlineStr"/>
+      <c r="K69" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L69" s="2" t="inlineStr"/>
+      <c r="M69" s="2" t="inlineStr">
+        <is>
+          <t>torso_haekelshirt_3.png</t>
+        </is>
+      </c>
+      <c r="N69" s="2" t="inlineStr">
+        <is>
+          <t>icon_torso_haekelshirt_3.png</t>
+        </is>
+      </c>
+      <c r="O69" s="2" t="inlineStr"/>
+      <c r="P69" s="2" t="inlineStr">
+        <is>
+          <t>Frau</t>
+        </is>
+      </c>
+      <c r="Q69" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R69" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 66</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>torso_ausgefranstesshirt_1</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>torso</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>Ausgefranstes Shirt</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I70" s="2" t="inlineStr"/>
+      <c r="J70" s="2" t="inlineStr"/>
+      <c r="K70" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L70" s="2" t="inlineStr"/>
+      <c r="M70" s="2" t="inlineStr">
+        <is>
+          <t>torso_ausgefranstesshirt_1.png</t>
+        </is>
+      </c>
+      <c r="N70" s="2" t="inlineStr">
+        <is>
+          <t>icon_torso_ausgefranstesshirt_1.png</t>
+        </is>
+      </c>
+      <c r="O70" s="2" t="inlineStr"/>
+      <c r="P70" s="2" t="inlineStr">
+        <is>
+          <t>Mann</t>
+        </is>
+      </c>
+      <c r="Q70" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R70" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 78</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>torso_tanktop_1</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>torso</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>Tanktop</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I71" s="2" t="inlineStr"/>
+      <c r="J71" s="2" t="inlineStr"/>
+      <c r="K71" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L71" s="2" t="inlineStr"/>
+      <c r="M71" s="2" t="inlineStr">
+        <is>
+          <t>torso_tanktop_1.png</t>
+        </is>
+      </c>
+      <c r="N71" s="2" t="inlineStr">
+        <is>
+          <t>icon_torso_tanktop_1.png</t>
+        </is>
+      </c>
+      <c r="O71" s="2" t="inlineStr"/>
+      <c r="P71" s="2" t="inlineStr">
+        <is>
+          <t>Mann</t>
+        </is>
+      </c>
+      <c r="Q71" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R71" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 85</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>schuhe_geflochtenesandalen_2</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>schuhe</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>Geflochtene Sandalen</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E72" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F72" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G72" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H72" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I72" s="2" t="inlineStr"/>
+      <c r="J72" s="2" t="inlineStr"/>
+      <c r="K72" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L72" s="2" t="inlineStr"/>
+      <c r="M72" s="2" t="inlineStr">
+        <is>
+          <t>schuhe_geflochtenesandalen_2.png</t>
+        </is>
+      </c>
+      <c r="N72" s="2" t="inlineStr">
+        <is>
+          <t>icon_schuhe_geflochtenesandalen_2.png</t>
+        </is>
+      </c>
+      <c r="O72" s="2" t="inlineStr"/>
+      <c r="P72" s="2" t="inlineStr">
+        <is>
+          <t>beide</t>
+        </is>
+      </c>
+      <c r="Q72" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R72" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 10</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>schuhe_riemensandalen_1</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>schuhe</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>Riemensandalen</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I73" s="2" t="inlineStr"/>
+      <c r="J73" s="2" t="inlineStr"/>
+      <c r="K73" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L73" s="2" t="inlineStr"/>
+      <c r="M73" s="2" t="inlineStr">
+        <is>
+          <t>schuhe_riemensandalen_1.png</t>
+        </is>
+      </c>
+      <c r="N73" s="2" t="inlineStr">
+        <is>
+          <t>icon_schuhe_riemensandalen_1.png</t>
+        </is>
+      </c>
+      <c r="O73" s="2" t="inlineStr"/>
+      <c r="P73" s="2" t="inlineStr">
+        <is>
+          <t>beide</t>
+        </is>
+      </c>
+      <c r="Q73" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R73" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 11</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>schuhe_knoechelsandalen_2</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>schuhe</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>Knöchelsandalen</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H74" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I74" s="2" t="inlineStr"/>
+      <c r="J74" s="2" t="inlineStr"/>
+      <c r="K74" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L74" s="2" t="inlineStr"/>
+      <c r="M74" s="2" t="inlineStr">
+        <is>
+          <t>schuhe_knoechelsandalen_2.png</t>
+        </is>
+      </c>
+      <c r="N74" s="2" t="inlineStr">
+        <is>
+          <t>icon_schuhe_knoechelsandalen_2.png</t>
+        </is>
+      </c>
+      <c r="O74" s="2" t="inlineStr"/>
+      <c r="P74" s="2" t="inlineStr">
+        <is>
+          <t>beide</t>
+        </is>
+      </c>
+      <c r="Q74" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R74" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 12</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>schuhe_zehensandalen_1</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>schuhe</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>Zehensandalen</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I75" s="2" t="inlineStr"/>
+      <c r="J75" s="2" t="inlineStr"/>
+      <c r="K75" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L75" s="2" t="inlineStr"/>
+      <c r="M75" s="2" t="inlineStr">
+        <is>
+          <t>schuhe_zehensandalen_1.png</t>
+        </is>
+      </c>
+      <c r="N75" s="2" t="inlineStr">
+        <is>
+          <t>icon_schuhe_zehensandalen_1.png</t>
+        </is>
+      </c>
+      <c r="O75" s="2" t="inlineStr"/>
+      <c r="P75" s="2" t="inlineStr">
+        <is>
+          <t>beide</t>
+        </is>
+      </c>
+      <c r="Q75" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R75" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 13</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>handschuhe_armwickel_2</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>handschuhe</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>Armwickel</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E76" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I76" s="2" t="inlineStr"/>
+      <c r="J76" s="2" t="inlineStr"/>
+      <c r="K76" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L76" s="2" t="inlineStr"/>
+      <c r="M76" s="2" t="inlineStr">
+        <is>
+          <t>handschuhe_armwickel_2.png</t>
+        </is>
+      </c>
+      <c r="N76" s="2" t="inlineStr">
+        <is>
+          <t>icon_handschuhe_armwickel_2.png</t>
+        </is>
+      </c>
+      <c r="O76" s="2" t="inlineStr"/>
+      <c r="P76" s="2" t="inlineStr">
+        <is>
+          <t>beide</t>
+        </is>
+      </c>
+      <c r="Q76" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R76" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 89, 95</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <dataValidations count="3">
+  <dataValidations count="5">
     <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"accessoire,beine,schuhe,torso,handschuhe,kopf"</formula1>
     </dataValidation>
     <dataValidation sqref="O2:O500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Hinter der Figur,Unter der Hose,Über den Schuhen,Über jeder Hose,Unter dem Oberteil,Über dem Oberteil,Ganz vorn"</formula1>
+    </dataValidation>
+    <dataValidation sqref="P2:P500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Frau,Mann,beide"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Q2:Q500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"ja,nein"</formula1>
     </dataValidation>
     <dataValidation sqref="E2:H500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="whole" operator="between">
       <formula1>0</formula1>
@@ -1738,7 +5438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1849,7 +5549,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Wie man das Teil bekommt, mit Komma getrennt: angezogen (trägt der Envoy von Anfang an), start (liegt beim Start im Rucksack), haendler, beute, quest.</t>
+          <t>Wie man das Teil bekommt, mit Komma getrennt: angezogen (trägt der Envoy von Anfang an), start (liegt beim Start im Rucksack), haendler, beute (von Geistern), fund (unterwegs gefunden, bei jeder Quest außer Bauen), quest.</t>
         </is>
       </c>
     </row>
@@ -1904,10 +5604,34 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>figur</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Für welche Figur die Zeichnung passt: Frau, Mann oder beide. Leer = beide. Die Fassung des Mannes liegt in assets/figur/zweite/; fehlt sie bei „beide“, trägt er die der Frau. Gefunden und angezogen werden kann ein Teil nur von der Figur, der es passt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>faerbbar</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>ja = jedes gefundene oder gekaufte Stück bekommt eine eigene Farbe (die App färbt die Zeichnung um, Haut bleibt). Leer oder nein = immer wie gezeichnet, etwa die Startkleidung und feste Questbelohnungen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>notiz</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>Nur für dich, erscheint nicht in der App.</t>
         </is>

</xml_diff>

<commit_message>
Kleidung: die drei Fußballtrikots als Fundstücke
Auf Wunsch der Nutzerin kommen die Trikots der Kleiderkammer (Nr. 54,
65 und 81, mit echten Logos; die App ist für die Familie) ins Spiel:
„Trikot mit der Acht“ für die Frau und „Trikot mit der Null“ für beide
Figuren, immer wie gezeichnet. Version 5.11.1.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0117M4aYJ5RoPwj7oU8m6XcB
</commit_message>
<xml_diff>
--- a/data/ausruestung.xlsx
+++ b/data/ausruestung.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R76"/>
+  <dimension ref="A1:R78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5406,6 +5406,138 @@
       <c r="R76" s="2" t="inlineStr">
         <is>
           <t>Kleiderkammer Nr. 89, 95</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>torso_trikotmitderacht_2</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>torso</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>Trikot mit der Acht</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E77" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I77" s="2" t="inlineStr"/>
+      <c r="J77" s="2" t="inlineStr"/>
+      <c r="K77" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L77" s="2" t="inlineStr"/>
+      <c r="M77" s="2" t="inlineStr">
+        <is>
+          <t>torso_trikotmitderacht_2.png</t>
+        </is>
+      </c>
+      <c r="N77" s="2" t="inlineStr">
+        <is>
+          <t>icon_torso_trikotmitderacht_2.png</t>
+        </is>
+      </c>
+      <c r="O77" s="2" t="inlineStr"/>
+      <c r="P77" s="2" t="inlineStr">
+        <is>
+          <t>Frau</t>
+        </is>
+      </c>
+      <c r="Q77" s="2" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="R77" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 54</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>torso_trikotmitdernull_2</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>torso</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>Trikot mit der Null</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F78" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I78" s="2" t="inlineStr"/>
+      <c r="J78" s="2" t="inlineStr"/>
+      <c r="K78" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L78" s="2" t="inlineStr"/>
+      <c r="M78" s="2" t="inlineStr">
+        <is>
+          <t>torso_trikotmitdernull_2.png</t>
+        </is>
+      </c>
+      <c r="N78" s="2" t="inlineStr">
+        <is>
+          <t>icon_torso_trikotmitdernull_2.png</t>
+        </is>
+      </c>
+      <c r="O78" s="2" t="inlineStr"/>
+      <c r="P78" s="2" t="inlineStr">
+        <is>
+          <t>beide</t>
+        </is>
+      </c>
+      <c r="Q78" s="2" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="R78" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 65, 81</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
5.20.6: Der Steppenrock, gezeichnet von der Tochter der Nutzerin
Neues Kleidungsstück für die Frau (Tabelle über den Generator, Ebene und
Icon aus ihrer Zeichnung, immer wie gezeichnet). Ab dem 8. Oktober hängt
er auf dem ersten Zettel am Aushang, mindestens selten, bis der Envoy ihn
hat (JOB_FEATURED); danach bleibt er als Fundstück im Spiel.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0117M4aYJ5RoPwj7oU8m6XcB
</commit_message>
<xml_diff>
--- a/data/ausruestung.xlsx
+++ b/data/ausruestung.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R78"/>
+  <dimension ref="A1:R79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5538,6 +5538,72 @@
       <c r="R78" s="2" t="inlineStr">
         <is>
           <t>Kleiderkammer Nr. 65, 81</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>beine_steppenrock_1</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>beine</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>Steppenrock</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I79" s="2" t="inlineStr"/>
+      <c r="J79" s="2" t="inlineStr"/>
+      <c r="K79" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L79" s="2" t="inlineStr"/>
+      <c r="M79" s="2" t="inlineStr">
+        <is>
+          <t>beine_steppenrock_1.png</t>
+        </is>
+      </c>
+      <c r="N79" s="2" t="inlineStr">
+        <is>
+          <t>icon_beine_steppenrock_1.png</t>
+        </is>
+      </c>
+      <c r="O79" s="2" t="inlineStr"/>
+      <c r="P79" s="2" t="inlineStr">
+        <is>
+          <t>Frau</t>
+        </is>
+      </c>
+      <c r="Q79" s="2" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="R79" s="2" t="inlineStr">
+        <is>
+          <t>gezeichnet von der Tochter der Nutzerin</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
5.20.11: Fliegerbrille, Lichterkette-Plan nur am 9. Oktober sicher
Neues Kopfteil Fliegerbrille (Kleiderkammer Nr. 97, für beide Figuren,
ohne Anforderung, als Fundstück). Der Plan der Lichterkette liegt am
9. Oktober 2026 sicher beim Händler, sonst mit Glück wie jeder Plan.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0117M4aYJ5RoPwj7oU8m6XcB
</commit_message>
<xml_diff>
--- a/data/ausruestung.xlsx
+++ b/data/ausruestung.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R79"/>
+  <dimension ref="A1:R80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5544,17 +5544,17 @@
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>beine_steppenrock_1</t>
+          <t>kopf_fliegerbrille_1</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>beine</t>
+          <t>kopf</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>Steppenrock</t>
+          <t>Fliegerbrille</t>
         </is>
       </c>
       <c r="D79" s="2" t="n">
@@ -5582,26 +5582,92 @@
       <c r="L79" s="2" t="inlineStr"/>
       <c r="M79" s="2" t="inlineStr">
         <is>
-          <t>beine_steppenrock_1.png</t>
+          <t>kopf_fliegerbrille_1.png</t>
         </is>
       </c>
       <c r="N79" s="2" t="inlineStr">
         <is>
-          <t>icon_beine_steppenrock_1.png</t>
+          <t>icon_kopf_fliegerbrille_1.png</t>
         </is>
       </c>
       <c r="O79" s="2" t="inlineStr"/>
       <c r="P79" s="2" t="inlineStr">
         <is>
+          <t>beide</t>
+        </is>
+      </c>
+      <c r="Q79" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="R79" s="2" t="inlineStr">
+        <is>
+          <t>Kleiderkammer Nr. 97</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>beine_steppenrock_1</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>beine</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>Steppenrock</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I80" s="2" t="inlineStr"/>
+      <c r="J80" s="2" t="inlineStr"/>
+      <c r="K80" s="2" t="inlineStr">
+        <is>
+          <t>fund, beute, haendler</t>
+        </is>
+      </c>
+      <c r="L80" s="2" t="inlineStr"/>
+      <c r="M80" s="2" t="inlineStr">
+        <is>
+          <t>beine_steppenrock_1.png</t>
+        </is>
+      </c>
+      <c r="N80" s="2" t="inlineStr">
+        <is>
+          <t>icon_beine_steppenrock_1.png</t>
+        </is>
+      </c>
+      <c r="O80" s="2" t="inlineStr"/>
+      <c r="P80" s="2" t="inlineStr">
+        <is>
           <t>Frau</t>
         </is>
       </c>
-      <c r="Q79" s="2" t="inlineStr">
+      <c r="Q80" s="2" t="inlineStr">
         <is>
           <t>nein</t>
         </is>
       </c>
-      <c r="R79" s="2" t="inlineStr">
+      <c r="R80" s="2" t="inlineStr">
         <is>
           <t>gezeichnet von der Tochter der Nutzerin</t>
         </is>

</xml_diff>